<commit_message>
feat: single-Excel multi-vendor workflow
- Add OLT Type column support for mixed ZTE/VSOL in one sheet
- config_generator.py now accepts templates directory, auto-selects per row
- Updated sample Excel with OLT Type column
- README rewritten to match real field workflow (list all sites in one Excel, run once)
</commit_message>
<xml_diff>
--- a/sample_data/sample_site_data.xlsx
+++ b/sample_data/sample_site_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,15 +429,20 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>OLT Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Private IP</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>TMVLAN</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>MVLAN</t>
         </is>
@@ -456,13 +461,18 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>ZTE GVGO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>10.100.1.1/22</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>800</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>900</v>
       </c>
     </row>
@@ -479,13 +489,18 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>ZTE GVGH</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>10.100.2.1/22</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>800</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>900</v>
       </c>
     </row>
@@ -502,13 +517,18 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>VSOL</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>10.100.3.1/22</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>801</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>901</v>
       </c>
     </row>
@@ -525,13 +545,18 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>ZTE GVGO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>10.101.1.1/22</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>800</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>900</v>
       </c>
     </row>
@@ -548,13 +573,18 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>VSOL</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>10.101.2.1/22</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>801</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>901</v>
       </c>
     </row>
@@ -571,13 +601,18 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>ZTE GVGH</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>10.102.1.1/22</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>800</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>900</v>
       </c>
     </row>
@@ -594,13 +629,18 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>ZTE GVGO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>10.102.2.1/22</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>800</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>900</v>
       </c>
     </row>
@@ -617,13 +657,18 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>VSOL</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>10.102.3.1/22</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>801</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>901</v>
       </c>
     </row>
@@ -640,13 +685,18 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>ZTE GVGO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>10.102.4.1/22</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>800</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>900</v>
       </c>
     </row>

</xml_diff>